<commit_message>
Update Block Reuse Summary sheet with page URLs
- Changed "Pages Used On" column to "Page URLs" with actual paths
- Added 3 additional blocks: Quick Links, Promo Banner, Video Hero
- Now shows 23 block types with their specific page URLs
- URLs enable direct navigation to see block in context

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/att-business-migration-plan.xlsx
+++ b/att-business-migration-plan.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="219">
   <si>
     <t>AT&amp;T Business Website Migration Plan</t>
   </si>
@@ -403,217 +403,220 @@
     <t>Page Count</t>
   </si>
   <si>
-    <t>Pages Used On</t>
+    <t>Page URLs</t>
   </si>
   <si>
     <t>Hero Blocks</t>
   </si>
   <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>/, /products/wireless-plans.html, /products/business-fiber-internet.html, /industries/healthcare.html, /portfolios/mobility.html, /learn/customer-stories/portx.html</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>/products/wireless-plans.html, /products/business-fiber-internet.html</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>/, /products/wireless-plans.html, /products/business-fiber-internet.html</t>
+  </si>
+  <si>
+    <t>/products/business-fiber-internet.html, /portfolios/mobility.html</t>
+  </si>
+  <si>
+    <t>/, /portfolios/mobility.html</t>
+  </si>
+  <si>
+    <t>/, /industries/healthcare.html, /products/business-fiber-internet.html</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Phase</t>
+  </si>
+  <si>
+    <t>Timeline</t>
+  </si>
+  <si>
+    <t>Goal</t>
+  </si>
+  <si>
+    <t>Tasks</t>
+  </si>
+  <si>
+    <t>Phase 1: Foundation</t>
+  </si>
+  <si>
+    <t>Weeks 1-2</t>
+  </si>
+  <si>
+    <t>Establish core infrastructure</t>
+  </si>
+  <si>
+    <t>Project Setup, Global Components, Base CSS, Pilot Page</t>
+  </si>
+  <si>
+    <t>Phase 2: Core Blocks</t>
+  </si>
+  <si>
+    <t>Weeks 3-5</t>
+  </si>
+  <si>
+    <t>Build reusable block library</t>
+  </si>
+  <si>
+    <t>Hero, Cards, Pricing, Lead Form, FAQ, Links, Video, Tabs</t>
+  </si>
+  <si>
+    <t>Phase 3: Page Templates</t>
+  </si>
+  <si>
+    <t>Weeks 6-8</t>
+  </si>
+  <si>
+    <t>Create primary page types</t>
+  </si>
+  <si>
+    <t>Homepage, Products, Portfolios, Industries, Categories</t>
+  </si>
+  <si>
+    <t>Phase 4: Content Migration</t>
+  </si>
+  <si>
+    <t>Weeks 9-12</t>
+  </si>
+  <si>
+    <t>Full content migration</t>
+  </si>
+  <si>
+    <t>Remaining Products, Customer Stories, Support pages</t>
+  </si>
+  <si>
+    <t>Phase 5: QA &amp; Launch</t>
+  </si>
+  <si>
+    <t>Weeks 13-14</t>
+  </si>
+  <si>
+    <t>Testing and go-live</t>
+  </si>
+  <si>
+    <t>Cross-browser, Mobile, Accessibility, Performance, Go-live</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Page Type</t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
+    <t>Justification</t>
+  </si>
+  <si>
+    <t>P1 - Critical</t>
+  </si>
+  <si>
+    <t>Primary entry point</t>
+  </si>
+  <si>
+    <t>Revenue driver</t>
+  </si>
+  <si>
+    <t>Top converting page</t>
+  </si>
+  <si>
+    <t>P2 - High</t>
+  </si>
+  <si>
+    <t>Product Pages (top 10)</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>High traffic products</t>
+  </si>
+  <si>
+    <t>Portfolio Pages</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>Category navigation</t>
+  </si>
+  <si>
+    <t>P3 - Medium</t>
+  </si>
+  <si>
+    <t>Industry Pages</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>Vertical targeting</t>
+  </si>
+  <si>
+    <t>Category Pages</t>
+  </si>
+  <si>
+    <t>18+</t>
+  </si>
+  <si>
+    <t>Product groupings</t>
+  </si>
+  <si>
+    <t>P4 - Lower</t>
+  </si>
+  <si>
+    <t>Customer Stories</t>
+  </si>
+  <si>
+    <t>27+</t>
+  </si>
+  <si>
+    <t>Supporting content</t>
+  </si>
+  <si>
+    <t>P5 - Lowest</t>
+  </si>
+  <si>
+    <t>Support/Utility</t>
+  </si>
+  <si>
     <t>5</t>
   </si>
   <si>
-    <t>Homepage, Wireless Plans, Business Fiber, Healthcare, Mobility, Customer Stories</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>Wireless Plans, Business Fiber</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>Homepage, Wireless Plans, Business Fiber</t>
-  </si>
-  <si>
-    <t>Business Fiber, Mobility Portfolio</t>
-  </si>
-  <si>
-    <t>Homepage, Mobility Portfolio</t>
-  </si>
-  <si>
-    <t>Homepage, Healthcare Industry, Business Fiber</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>Industry Pages</t>
-  </si>
-  <si>
-    <t>Customer Stories</t>
+    <t>Low change frequency</t>
+  </si>
+  <si>
+    <t>% of Total</t>
+  </si>
+  <si>
+    <t>Est. Count</t>
+  </si>
+  <si>
+    <t>Content/Articles</t>
+  </si>
+  <si>
+    <t>40%</t>
+  </si>
+  <si>
+    <t>~300</t>
   </si>
   <si>
     <t>Product Pages</t>
-  </si>
-  <si>
-    <t>Phase</t>
-  </si>
-  <si>
-    <t>Timeline</t>
-  </si>
-  <si>
-    <t>Goal</t>
-  </si>
-  <si>
-    <t>Tasks</t>
-  </si>
-  <si>
-    <t>Phase 1: Foundation</t>
-  </si>
-  <si>
-    <t>Weeks 1-2</t>
-  </si>
-  <si>
-    <t>Establish core infrastructure</t>
-  </si>
-  <si>
-    <t>Project Setup, Global Components, Base CSS, Pilot Page</t>
-  </si>
-  <si>
-    <t>Phase 2: Core Blocks</t>
-  </si>
-  <si>
-    <t>Weeks 3-5</t>
-  </si>
-  <si>
-    <t>Build reusable block library</t>
-  </si>
-  <si>
-    <t>Hero, Cards, Pricing, Lead Form, FAQ, Links, Video, Tabs</t>
-  </si>
-  <si>
-    <t>Phase 3: Page Templates</t>
-  </si>
-  <si>
-    <t>Weeks 6-8</t>
-  </si>
-  <si>
-    <t>Create primary page types</t>
-  </si>
-  <si>
-    <t>Homepage, Products, Portfolios, Industries, Categories</t>
-  </si>
-  <si>
-    <t>Phase 4: Content Migration</t>
-  </si>
-  <si>
-    <t>Weeks 9-12</t>
-  </si>
-  <si>
-    <t>Full content migration</t>
-  </si>
-  <si>
-    <t>Remaining Products, Customer Stories, Support pages</t>
-  </si>
-  <si>
-    <t>Phase 5: QA &amp; Launch</t>
-  </si>
-  <si>
-    <t>Weeks 13-14</t>
-  </si>
-  <si>
-    <t>Testing and go-live</t>
-  </si>
-  <si>
-    <t>Cross-browser, Mobile, Accessibility, Performance, Go-live</t>
-  </si>
-  <si>
-    <t>Priority</t>
-  </si>
-  <si>
-    <t>Page Type</t>
-  </si>
-  <si>
-    <t>Count</t>
-  </si>
-  <si>
-    <t>Justification</t>
-  </si>
-  <si>
-    <t>P1 - Critical</t>
-  </si>
-  <si>
-    <t>Primary entry point</t>
-  </si>
-  <si>
-    <t>Revenue driver</t>
-  </si>
-  <si>
-    <t>Top converting page</t>
-  </si>
-  <si>
-    <t>P2 - High</t>
-  </si>
-  <si>
-    <t>Product Pages (top 10)</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>High traffic products</t>
-  </si>
-  <si>
-    <t>Portfolio Pages</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>Category navigation</t>
-  </si>
-  <si>
-    <t>P3 - Medium</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>Vertical targeting</t>
-  </si>
-  <si>
-    <t>Category Pages</t>
-  </si>
-  <si>
-    <t>18+</t>
-  </si>
-  <si>
-    <t>Product groupings</t>
-  </si>
-  <si>
-    <t>P4 - Lower</t>
-  </si>
-  <si>
-    <t>27+</t>
-  </si>
-  <si>
-    <t>Supporting content</t>
-  </si>
-  <si>
-    <t>P5 - Lowest</t>
-  </si>
-  <si>
-    <t>Support/Utility</t>
-  </si>
-  <si>
-    <t>Low change frequency</t>
-  </si>
-  <si>
-    <t>% of Total</t>
-  </si>
-  <si>
-    <t>Est. Count</t>
-  </si>
-  <si>
-    <t>Content/Articles</t>
-  </si>
-  <si>
-    <t>40%</t>
-  </si>
-  <si>
-    <t>~300</t>
   </si>
   <si>
     <t>20%</t>
@@ -723,10 +726,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -3328,12 +3334,12 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="60" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="90" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3354,7 +3360,7 @@
       <c r="B2" t="s">
         <v>130</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="3" t="s">
         <v>131</v>
       </c>
     </row>
@@ -3365,7 +3371,7 @@
       <c r="B3" t="s">
         <v>132</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="3" t="s">
         <v>133</v>
       </c>
     </row>
@@ -3376,7 +3382,7 @@
       <c r="B4" t="s">
         <v>134</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="3" t="s">
         <v>135</v>
       </c>
     </row>
@@ -3387,7 +3393,7 @@
       <c r="B5" t="s">
         <v>132</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="3" t="s">
         <v>136</v>
       </c>
     </row>
@@ -3398,7 +3404,7 @@
       <c r="B6" t="s">
         <v>132</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="3" t="s">
         <v>137</v>
       </c>
     </row>
@@ -3409,7 +3415,7 @@
       <c r="B7" t="s">
         <v>132</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="3" t="s">
         <v>133</v>
       </c>
     </row>
@@ -3420,7 +3426,7 @@
       <c r="B8" t="s">
         <v>134</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="3" t="s">
         <v>138</v>
       </c>
     </row>
@@ -3431,8 +3437,8 @@
       <c r="B9" t="s">
         <v>139</v>
       </c>
-      <c r="C9" t="s">
-        <v>50</v>
+      <c r="C9" s="3" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -3442,8 +3448,8 @@
       <c r="B10" t="s">
         <v>139</v>
       </c>
-      <c r="C10" t="s">
-        <v>50</v>
+      <c r="C10" s="3" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -3453,8 +3459,8 @@
       <c r="B11" t="s">
         <v>139</v>
       </c>
-      <c r="C11" t="s">
-        <v>50</v>
+      <c r="C11" s="3" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -3464,8 +3470,8 @@
       <c r="B12" t="s">
         <v>139</v>
       </c>
-      <c r="C12" t="s">
-        <v>140</v>
+      <c r="C12" s="3" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -3475,8 +3481,8 @@
       <c r="B13" t="s">
         <v>139</v>
       </c>
-      <c r="C13" t="s">
-        <v>140</v>
+      <c r="C13" s="3" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -3486,8 +3492,8 @@
       <c r="B14" t="s">
         <v>139</v>
       </c>
-      <c r="C14" t="s">
-        <v>140</v>
+      <c r="C14" s="3" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -3497,8 +3503,8 @@
       <c r="B15" t="s">
         <v>139</v>
       </c>
-      <c r="C15" t="s">
-        <v>140</v>
+      <c r="C15" s="3" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -3508,8 +3514,8 @@
       <c r="B16" t="s">
         <v>139</v>
       </c>
-      <c r="C16" t="s">
-        <v>140</v>
+      <c r="C16" s="3" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -3519,8 +3525,8 @@
       <c r="B17" t="s">
         <v>139</v>
       </c>
-      <c r="C17" t="s">
-        <v>140</v>
+      <c r="C17" s="3" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -3530,8 +3536,8 @@
       <c r="B18" t="s">
         <v>139</v>
       </c>
-      <c r="C18" t="s">
-        <v>141</v>
+      <c r="C18" s="3" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -3541,8 +3547,8 @@
       <c r="B19" t="s">
         <v>139</v>
       </c>
-      <c r="C19" t="s">
-        <v>141</v>
+      <c r="C19" s="3" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -3552,8 +3558,8 @@
       <c r="B20" t="s">
         <v>139</v>
       </c>
-      <c r="C20" t="s">
-        <v>142</v>
+      <c r="C20" s="3" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -3563,8 +3569,41 @@
       <c r="B21" t="s">
         <v>139</v>
       </c>
-      <c r="C21" t="s">
-        <v>142</v>
+      <c r="C21" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>49</v>
+      </c>
+      <c r="B22" t="s">
+        <v>139</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>54</v>
+      </c>
+      <c r="B23" t="s">
+        <v>139</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>58</v>
+      </c>
+      <c r="B24" t="s">
+        <v>139</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -3586,86 +3625,86 @@
   <sheetData>
     <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>143</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D2" t="s">
         <v>147</v>
-      </c>
-      <c r="B2" t="s">
-        <v>148</v>
-      </c>
-      <c r="C2" t="s">
-        <v>149</v>
-      </c>
-      <c r="D2" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>148</v>
+      </c>
+      <c r="B3" t="s">
+        <v>149</v>
+      </c>
+      <c r="C3" t="s">
+        <v>150</v>
+      </c>
+      <c r="D3" t="s">
         <v>151</v>
-      </c>
-      <c r="B3" t="s">
-        <v>152</v>
-      </c>
-      <c r="C3" t="s">
-        <v>153</v>
-      </c>
-      <c r="D3" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>152</v>
+      </c>
+      <c r="B4" t="s">
+        <v>153</v>
+      </c>
+      <c r="C4" t="s">
+        <v>154</v>
+      </c>
+      <c r="D4" t="s">
         <v>155</v>
-      </c>
-      <c r="B4" t="s">
-        <v>156</v>
-      </c>
-      <c r="C4" t="s">
-        <v>157</v>
-      </c>
-      <c r="D4" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>156</v>
+      </c>
+      <c r="B5" t="s">
+        <v>157</v>
+      </c>
+      <c r="C5" t="s">
+        <v>158</v>
+      </c>
+      <c r="D5" t="s">
         <v>159</v>
-      </c>
-      <c r="B5" t="s">
-        <v>160</v>
-      </c>
-      <c r="C5" t="s">
-        <v>161</v>
-      </c>
-      <c r="D5" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>160</v>
+      </c>
+      <c r="B6" t="s">
+        <v>161</v>
+      </c>
+      <c r="C6" t="s">
+        <v>162</v>
+      </c>
+      <c r="D6" t="s">
         <v>163</v>
-      </c>
-      <c r="B6" t="s">
-        <v>164</v>
-      </c>
-      <c r="C6" t="s">
-        <v>165</v>
-      </c>
-      <c r="D6" t="s">
-        <v>166</v>
       </c>
     </row>
   </sheetData>
@@ -3687,21 +3726,21 @@
   <sheetData>
     <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>167</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B2" t="s">
         <v>50</v>
@@ -3710,12 +3749,12 @@
         <v>139</v>
       </c>
       <c r="D2" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B3" t="s">
         <v>39</v>
@@ -3724,12 +3763,12 @@
         <v>139</v>
       </c>
       <c r="D3" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B4" t="s">
         <v>61</v>
@@ -3738,88 +3777,88 @@
         <v>139</v>
       </c>
       <c r="D4" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>172</v>
+      </c>
+      <c r="B5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C5" t="s">
+        <v>174</v>
+      </c>
+      <c r="D5" t="s">
         <v>175</v>
-      </c>
-      <c r="B5" t="s">
-        <v>176</v>
-      </c>
-      <c r="C5" t="s">
-        <v>177</v>
-      </c>
-      <c r="D5" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="B6" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="C6" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="D6" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>179</v>
+      </c>
+      <c r="B7" t="s">
+        <v>180</v>
+      </c>
+      <c r="C7" t="s">
+        <v>181</v>
+      </c>
+      <c r="D7" t="s">
         <v>182</v>
-      </c>
-      <c r="B7" t="s">
-        <v>140</v>
-      </c>
-      <c r="C7" t="s">
-        <v>183</v>
-      </c>
-      <c r="D7" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="B8" t="s">
+        <v>183</v>
+      </c>
+      <c r="C8" t="s">
+        <v>184</v>
+      </c>
+      <c r="D8" t="s">
         <v>185</v>
-      </c>
-      <c r="C8" t="s">
-        <v>186</v>
-      </c>
-      <c r="D8" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>186</v>
+      </c>
+      <c r="B9" t="s">
+        <v>187</v>
+      </c>
+      <c r="C9" t="s">
         <v>188</v>
       </c>
-      <c r="B9" t="s">
-        <v>141</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>189</v>
-      </c>
-      <c r="D9" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>190</v>
+      </c>
+      <c r="B10" t="s">
         <v>191</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>192</v>
-      </c>
-      <c r="C10" t="s">
-        <v>130</v>
       </c>
       <c r="D10" t="s">
         <v>193</v>
@@ -3842,7 +3881,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>194</v>
@@ -3864,68 +3903,68 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>142</v>
+        <v>199</v>
       </c>
       <c r="B3" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>141</v>
+        <v>187</v>
       </c>
       <c r="B4" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C4" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B5" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C5" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B7" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C7" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C8" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -3939,15 +3978,15 @@
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="B10" s="3" t="s">
+    <row r="10" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="B10" s="4" t="s">
         <v>217</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>218</v>
       </c>
     </row>
   </sheetData>

</xml_diff>